<commit_message>
Recompute sales-by-price-tier summary with updated tier assignments
Source sheet's 온라인/오프라인 가격대(고/중/저) tags changed for
several models (e.g. SHP-DP951MC, SHP-P52HCXC, ZD-P61-FNXS moved
from 고 to 중; SHP-P52SCXC moved from 고/중 to 중/중). Re-pulled the
sheet and recomputed both tables; totals re-verified against the
sheet's own 계 row for all 7 months.
</commit_message>
<xml_diff>
--- a/온라인오프라인_가격대별_판매수량_1-7월.xlsx
+++ b/온라인오프라인_가격대별_판매수량_1-7월.xlsx
@@ -564,25 +564,25 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I5" s="5">
         <f>SUM(B5:H5)</f>
@@ -596,25 +596,25 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>961</v>
+        <v>968</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1363</v>
+        <v>1368</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>1510</v>
+        <v>1512</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="I6" s="5">
         <f>SUM(B6:H6)</f>
@@ -797,25 +797,25 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2042</v>
+        <v>616</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>1200</v>
+        <v>700</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>1250</v>
+        <v>550</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>856</v>
+        <v>748</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>540</v>
+        <v>440</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>792</v>
+        <v>652</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>1253</v>
+        <v>1213</v>
       </c>
       <c r="I5" s="5">
         <f>SUM(B5:H5)</f>
@@ -829,25 +829,25 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1681</v>
+        <v>3707</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2052</v>
+        <v>2952</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>950</v>
+        <v>1850</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>740</v>
+        <v>1148</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>460</v>
+        <v>1012</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>552</v>
+        <v>1144</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>522</v>
+        <v>1163</v>
       </c>
       <c r="I6" s="5">
         <f>SUM(B6:H6)</f>
@@ -861,25 +861,25 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2050</v>
+        <v>1450</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1900</v>
+        <v>1500</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>2300</v>
+        <v>2100</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>1692</v>
+        <v>1240</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>1252</v>
+        <v>800</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>1533</v>
+        <v>932</v>
       </c>
       <c r="I7" s="5">
         <f>SUM(B7:H7)</f>

</xml_diff>

<commit_message>
Recompute offline sales-by-price-tier with latest tier assignments
Source sheet's 오프라인 가격대 tags changed again (e.g. SHP-DP951MC,
ZD-P61-FNXS moved back to 고). Online tiers unchanged this round.
Totals re-verified against the sheet's own 계 row for all 7 months.
</commit_message>
<xml_diff>
--- a/온라인오프라인_가격대별_판매수량_1-7월.xlsx
+++ b/온라인오프라인_가격대별_판매수량_1-7월.xlsx
@@ -797,16 +797,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>616</v>
+        <v>1452</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>550</v>
+        <v>750</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>748</v>
+        <v>756</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>440</v>
@@ -829,16 +829,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>3707</v>
+        <v>2871</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2952</v>
+        <v>2852</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1850</v>
+        <v>1650</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1148</v>
+        <v>1140</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>1012</v>

</xml_diff>

<commit_message>
Recompute sales-by-price-tier again after another tier reclassification
SHP-P52HCXC moved back to 고/고 (was 중/중); resulting online tiers
match the original run, offline 중 changed. Verified against 계 row.
</commit_message>
<xml_diff>
--- a/온라인오프라인_가격대별_판매수량_1-7월.xlsx
+++ b/온라인오프라인_가격대별_판매수량_1-7월.xlsx
@@ -564,25 +564,25 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I5" s="5">
         <f>SUM(B5:H5)</f>
@@ -596,25 +596,25 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>761</v>
+        <v>754</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>968</v>
+        <v>961</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1368</v>
+        <v>1363</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>1512</v>
+        <v>1510</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="I6" s="5">
         <f>SUM(B6:H6)</f>
@@ -797,25 +797,25 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1452</v>
+        <v>2042</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>756</v>
+        <v>856</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>440</v>
+        <v>540</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>652</v>
+        <v>792</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>1213</v>
+        <v>1253</v>
       </c>
       <c r="I5" s="5">
         <f>SUM(B5:H5)</f>
@@ -829,25 +829,25 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>2871</v>
+        <v>2281</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2852</v>
+        <v>2452</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1650</v>
+        <v>1150</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1140</v>
+        <v>1040</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1012</v>
+        <v>912</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>1144</v>
+        <v>1004</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1163</v>
+        <v>1123</v>
       </c>
       <c r="I6" s="5">
         <f>SUM(B6:H6)</f>

</xml_diff>